<commit_message>
Proposition : rangée de bulles « Pour qui ? » au-dessus des jours (colonne Cibles), fiches inchangées
Colonne facultative Cibles (liste de choix) dans Evenements, remplie d'après les
quatre plannings PDF (Pédagogie 13, Recherche 16, Étudiants 7, Entreprises 13).
Une rangée de bulles au-dessus des jours, plusieurs publics possibles, rien sur
les fiches ni dans les onglets, choix mémorisé sur l'appareil. Sans colonne
Cibles, le widget ne change pas. Tests : unitaires, faux Grist et vrai Grist.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FPLB4wrip8pBNBGYDq5d2D
</commit_message>
<xml_diff>
--- a/data/Evenements_Semaine_Innovation_2026.xlsx
+++ b/data/Evenements_Semaine_Innovation_2026.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evenements" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Evenements'!$A$1:$M$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Evenements'!$A$1:$N$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M31"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -459,8 +459,9 @@
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="44" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="70" customWidth="1" min="12" max="12"/>
-    <col width="60" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="70" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -521,10 +522,15 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Cibles</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Lien</t>
         </is>
@@ -576,12 +582,17 @@
           <t>Enseignants-chercheurs, doctorants</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>Pédagogie, Recherche</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>Initiation au Transmedia Storytelling : concevoir en groupe une stratégie de récits multiplateformes pour valoriser un projet.</t>
         </is>
       </c>
-      <c r="M2" s="5" t="inlineStr">
+      <c r="N2" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/le-transmedia-storytelling-comme-valorisation-de-projets</t>
         </is>
@@ -633,12 +644,17 @@
           <t>Personnels</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Pédagogie, Recherche</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>Jeux de société détournés et défis de créativité pour découvrir les méthodes de l’innovation de façon ludique, sans prérequis.</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="N3" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/les-dejeuxners-de-linnovation</t>
         </is>
@@ -694,12 +710,17 @@
           <t>Enseignants-chercheurs, chercheurs, personnels, étudiants</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Pédagogie, Étudiants</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>Outils ludiques (jeu de société collaboratif, calculateur Ecobalyse) pour évaluer l’empreinte environnementale de produits.</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/evaluer-pour-mieux-maitriser-les-impacts-environnementaux</t>
         </is>
@@ -751,12 +772,17 @@
           <t>Enseignants-chercheurs, accompagnants pédagogiques</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Pédagogie</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>Atelier de co-conception pour imaginer des espaces d’apprentissage innovants et inclusifs, à partir de scénarios pédagogiques concrets.</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/construisons-ensemble-un-espace-pour-apprendre-autrement</t>
         </is>
@@ -804,8 +830,13 @@
           <t>Grand public</t>
         </is>
       </c>
-      <c r="L6" s="4" t="n"/>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>Pédagogie, Recherche, Étudiants, Entreprises</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/semaine-de-linnovation-2026-3e-edition</t>
         </is>
@@ -857,12 +888,17 @@
           <t>Enseignants-chercheurs, chercheurs, doctorants, étudiants de master</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>Recherche</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>Des binômes chercheur / industriel partagent leurs retours sur leurs collaborations ; présentation des dispositifs pour monter et financer des projets communs.</t>
         </is>
       </c>
-      <c r="M7" s="5" t="inlineStr">
+      <c r="N7" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/entractes-regards-croises-sur-les-collaborations-entre-recherche-academique-en-sante-et-entreprise</t>
         </is>
@@ -918,12 +954,17 @@
           <t>Enseignants-chercheurs, acteurs socio-économiques</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Recherche, Entreprises</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>Matinée organisée par NOBATEK et l’université de Bordeaux (équipe GP2E) sur la performance énergétique et environnementale des bâtiments.</t>
         </is>
       </c>
-      <c r="M8" s="5" t="inlineStr">
+      <c r="N8" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/matinale-scientifique-garantie-de-performances-energetiques-et-environnementales-des-batiments</t>
         </is>
@@ -975,12 +1016,17 @@
           <t>Étudiants, personnels, acteurs socio-économiques</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Étudiants, Entreprises</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>Journée de présentations, témoignages et échanges sur les dispositifs d’appui à l’entrepreneuriat agricole et agroalimentaire, avec visite de la plateforme FarmLab@Bordeaux.</t>
         </is>
       </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="N9" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/un-terrain-fertile-pour-lentrepreneuriat-et-linnovation-au-service-des-transitions-agroecologiques</t>
         </is>
@@ -1032,12 +1078,17 @@
           <t>Enseignants-chercheurs, ingénieurs, professionnels de la formation</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Pédagogie</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>Visite de la Learning Factory des Arts et Métiers : des plateformes pédagogiques proches de l’industrie, du prototypage à la production mécanique.</t>
         </is>
       </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="N10" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/les-evolutive-learning-factories-des-usines-ecoles-pour-apprendre-autrement</t>
         </is>
@@ -1085,12 +1136,17 @@
           <t>Étudiants</t>
         </is>
       </c>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Étudiants</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>Jeux de société détournés et défis de créativité pour découvrir les méthodes de l’innovation de façon ludique, sans prérequis.</t>
         </is>
       </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="N11" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/les-dejeuxners-de-linnovation</t>
         </is>
@@ -1138,12 +1194,17 @@
           <t>Acteurs socio-économiques</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Entreprises</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t>Visite commentée du CATIE, centre de ressources technologiques du numérique : expertises, équipements et projets menés avec des entreprises.</t>
         </is>
       </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="N12" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/de-la-recheche-linnovation-concrete-en-entreprise-la-valeur-ajoutee-dun-centre-de-ressources-technologiques-comme-le-catie</t>
         </is>
@@ -1195,12 +1256,17 @@
           <t>Architectes, ingénieurs, chercheurs, étudiants, professionnels de la construction et de la filière bois</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>Recherche, Étudiants, Entreprises</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>Visite des démonstrateurs THRIVE et TNEB : construire avec le hêtre et les feuillus locaux, la terre-paille et le chanvre. Départs des visites à 16 h et 17 h.</t>
         </is>
       </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="N13" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/construire-autrement-avec-le-hetre-la-terre-paille-et-le-chanvre</t>
         </is>
@@ -1256,12 +1322,17 @@
           <t>Étudiants et doctorants en sciences humaines et sociales</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Recherche, Étudiants</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>Soirée en trois temps : table ronde, atelier collaboratif et pitchs d’étudiants autour de l’innovation en SHS.</t>
         </is>
       </c>
-      <c r="M14" s="5" t="inlineStr">
+      <c r="N14" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/mardis-de-lentrepreneuriat-les-sciences-humaines-et-sociales-moteur-dinnovation</t>
         </is>
@@ -1317,12 +1388,17 @@
           <t>Chercheurs en sciences humaines et sociales</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>Recherche, Entreprises</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
         <is>
           <t>Transformer une première collaboration avec un acteur socio-économique en partenariat durable : témoignages et échanges avec des experts.</t>
         </is>
       </c>
-      <c r="M15" s="5" t="inlineStr">
+      <c r="N15" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/faire-grandir-ses-partenariats-construire-des-collaborations-structurantes-en-sciences-humaines-et-sociales</t>
         </is>
@@ -1374,12 +1450,17 @@
           <t>Chercheurs du numérique, personnels de la valorisation, acteurs socio-économiques</t>
         </is>
       </c>
-      <c r="L16" s="4" t="inlineStr">
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Recherche, Entreprises</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
         <is>
           <t>Valoriser les logiciels de recherche en Open Source : visibilité, collaborations avec les entreprises, modèles économiques, licences.</t>
         </is>
       </c>
-      <c r="M16" s="5" t="inlineStr">
+      <c r="N16" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/du-laboratoire-lentreprise-le-potentiel-de-lopen-source-issu-de-la-recherche</t>
         </is>
@@ -1431,12 +1512,17 @@
           <t>Chercheurs, enseignants-chercheurs, industriels</t>
         </is>
       </c>
-      <c r="L17" s="4" t="inlineStr">
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>Recherche, Entreprises</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
         <is>
           <t>Journée autour des équipements de micro et nanofabrication du site bordelais pour définir une feuille de route technologique en photonique.</t>
         </is>
       </c>
-      <c r="M17" s="5" t="inlineStr">
+      <c r="N17" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/micro-et-nanofabrication-pour-la-photonique-avancee</t>
         </is>
@@ -1488,12 +1574,17 @@
           <t>Acteurs socio-économiques du secteur spatial</t>
         </is>
       </c>
-      <c r="L18" s="4" t="inlineStr">
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Entreprises</t>
+        </is>
+      </c>
+      <c r="M18" s="4" t="inlineStr">
         <is>
           <t>Découvrir les expertises, laboratoires et plateformes spatiales de l’université de Bordeaux, puis échanger avec les chercheurs (avec Aerospace Valley).</t>
         </is>
       </c>
-      <c r="M18" s="5" t="inlineStr">
+      <c r="N18" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/explorer-lespace-avec-nos-experts</t>
         </is>
@@ -1545,12 +1636,17 @@
           <t>Enseignants-chercheurs, chercheurs, acteurs socio-économiques</t>
         </is>
       </c>
-      <c r="L19" s="4" t="inlineStr">
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Recherche, Entreprises</t>
+        </is>
+      </c>
+      <c r="M19" s="4" t="inlineStr">
         <is>
           <t>Les coulisses des collaborations laboratoires-entreprises et le rôle des cellules de transfert technologique.</t>
         </is>
       </c>
-      <c r="M19" s="5" t="inlineStr">
+      <c r="N19" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/les-cellules-de-transfert-technologique-en-pratique</t>
         </is>
@@ -1610,12 +1706,17 @@
           <t>Acteurs socio-économiques (start-ups, deeptech, PME, ETI)</t>
         </is>
       </c>
-      <c r="L20" s="4" t="inlineStr">
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>Entreprises</t>
+        </is>
+      </c>
+      <c r="M20" s="4" t="inlineStr">
         <is>
           <t>Rencontrer les plateformes technologiques de l’université de Bordeaux et découvrir leurs équipements et compétences.</t>
         </is>
       </c>
-      <c r="M20" s="5" t="inlineStr">
+      <c r="N20" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/salon-des-entreprises-du-concept-au-demonstrateur</t>
         </is>
@@ -1667,12 +1768,17 @@
           <t>Enseignants-chercheurs, chercheurs, acteurs socio-économiques</t>
         </is>
       </c>
-      <c r="L21" s="4" t="inlineStr">
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Recherche</t>
+        </is>
+      </c>
+      <c r="M21" s="4" t="inlineStr">
         <is>
           <t>Rencontres entre chercheurs du GIS Albatros et industriels pour identifier des sujets communs (micro-projets, études, thèses CIFRE).</t>
         </is>
       </c>
-      <c r="M21" s="5" t="inlineStr">
+      <c r="N21" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/albatros-techno-day-2026</t>
         </is>
@@ -1728,12 +1834,17 @@
           <t>Enseignants-chercheurs</t>
         </is>
       </c>
-      <c r="L22" s="4" t="inlineStr">
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>Pédagogie</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
         <is>
           <t>Présentation de la plateforme CampusIABordeaux et de son usage avec les étudiants : publication, partage et réutilisation des données.</t>
         </is>
       </c>
-      <c r="M22" s="5" t="inlineStr">
+      <c r="N22" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/campusiabordeaux-entrainez-vos-etudiants-sur-la-donnee</t>
         </is>
@@ -1789,12 +1900,17 @@
           <t>Enseignants-chercheurs</t>
         </is>
       </c>
-      <c r="L23" s="4" t="inlineStr">
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>Pédagogie</t>
+        </is>
+      </c>
+      <c r="M23" s="4" t="inlineStr">
         <is>
           <t>Présentation du dispositif qui accompagne des projets d’acteurs de la société et co-construit des questions de recherche. Accueil café à 10 h 30, atelier à 10 h 45.</t>
         </is>
       </c>
-      <c r="M23" s="5" t="inlineStr">
+      <c r="N23" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/echoppe-des-sciences-decouvrez-questionnez-adoptez</t>
         </is>
@@ -1842,12 +1958,17 @@
           <t>Étudiants</t>
         </is>
       </c>
-      <c r="L24" s="4" t="inlineStr">
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>Étudiants</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
         <is>
           <t>Jeux de société détournés et défis de créativité pour découvrir les méthodes de l’innovation de façon ludique, sans prérequis.</t>
         </is>
       </c>
-      <c r="M24" s="5" t="inlineStr">
+      <c r="N24" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/les-dejeuxners-de-linnovation</t>
         </is>
@@ -1903,12 +2024,17 @@
           <t>Chercheurs, enseignants-chercheurs, doctorants</t>
         </is>
       </c>
-      <c r="L25" s="4" t="inlineStr">
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>Pédagogie, Recherche</t>
+        </is>
+      </c>
+      <c r="M25" s="4" t="inlineStr">
         <is>
           <t>Visite du FabLabNab (impression 3D, découpe laser, prototypage rapide) et temps d’échange sur la science ouverte et l’innovation frugale.</t>
         </is>
       </c>
-      <c r="M25" s="5" t="inlineStr">
+      <c r="N25" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/pepiniere-numerique-fablabnab-quand-la-fabrication-numerique-booste-linnovation</t>
         </is>
@@ -1960,12 +2086,17 @@
           <t>Enseignants-chercheurs, chercheurs, ingénieurs, doctorants, acteurs socio-économiques</t>
         </is>
       </c>
-      <c r="L26" s="4" t="inlineStr">
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>Pédagogie, Recherche, Entreprises</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
         <is>
           <t>Présentation-visite d’une cellule robotisée de fabrication additive métallique (WAAM) : fonctionnement, usages industriels et défis.</t>
         </is>
       </c>
-      <c r="M26" s="5" t="inlineStr">
+      <c r="N26" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/la-robotique-au-service-de-la-fabrication-additive-metallique</t>
         </is>
@@ -2017,12 +2148,17 @@
           <t>Docteurs et doctorants</t>
         </is>
       </c>
-      <c r="L27" s="4" t="inlineStr">
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>Recherche, Entreprises</t>
+        </is>
+      </c>
+      <c r="M27" s="4" t="inlineStr">
         <is>
           <t>Soirée de rencontre entre docteurs, doctorants et entreprises bordelaises : témoignages, échanges en petits groupes et réseautage.</t>
         </is>
       </c>
-      <c r="M27" s="5" t="inlineStr">
+      <c r="N27" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/afterwork-docteurs-doctorants-et-entreprises</t>
         </is>
@@ -2078,12 +2214,17 @@
           <t>Enseignants-chercheurs</t>
         </is>
       </c>
-      <c r="L28" s="4" t="inlineStr">
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>Pédagogie</t>
+        </is>
+      </c>
+      <c r="M28" s="4" t="inlineStr">
         <is>
           <t>Présentation de la plateforme CampusIABordeaux et de son usage avec les étudiants : publication, partage et réutilisation des données.</t>
         </is>
       </c>
-      <c r="M28" s="5" t="inlineStr">
+      <c r="N28" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/campusiabordeaux-entrainez-vos-etudiants-sur-la-donnee</t>
         </is>
@@ -2135,12 +2276,17 @@
           <t>Accompagnants à l’innovation, enseignants-chercheurs</t>
         </is>
       </c>
-      <c r="L29" s="4" t="inlineStr">
+      <c r="L29" s="5" t="inlineStr">
+        <is>
+          <t>Pédagogie, Recherche</t>
+        </is>
+      </c>
+      <c r="M29" s="4" t="inlineStr">
         <is>
           <t>Trois retours d’expérience sur des formations-accompagnements conçus sur mesure pour répondre à des besoins collectifs.</t>
         </is>
       </c>
-      <c r="M29" s="5" t="inlineStr">
+      <c r="N29" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/des-formations-sur-mesure-pour-faire-evoluer-ses-pratiques</t>
         </is>
@@ -2192,12 +2338,13 @@
           <t>Personnels administratifs</t>
         </is>
       </c>
-      <c r="L30" s="4" t="inlineStr">
+      <c r="L30" s="5" t="n"/>
+      <c r="M30" s="4" t="inlineStr">
         <is>
           <t>Jeu en équipes de 4 à 5 personnes pour tester sa connaissance de l’écosystème d’innovation bordelais et savoir orienter les porteurs de projets.</t>
         </is>
       </c>
-      <c r="M30" s="5" t="inlineStr">
+      <c r="N30" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/le-pole-universitaire-dinnovation-bordeaux-en-jeu-venez-relever-le-defi</t>
         </is>
@@ -2253,19 +2400,24 @@
           <t>Enseignants-chercheurs</t>
         </is>
       </c>
-      <c r="L31" s="4" t="inlineStr">
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>Pédagogie</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="inlineStr">
         <is>
           <t>Présentation de la plateforme CampusIABordeaux et de son usage avec les étudiants : publication, partage et réutilisation des données.</t>
         </is>
       </c>
-      <c r="M31" s="5" t="inlineStr">
+      <c r="N31" s="5" t="inlineStr">
         <is>
           <t>https://www.u-bordeaux.fr/evenements/campusiabordeaux-entrainez-vos-etudiants-sur-la-donnee</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M31"/>
+  <autoFilter ref="A1:N31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Filtre « Pour qui ? » : cinquième public « Personnels » (serious game), version « l »
Le serious game « No wrong door » n'est surligné sur aucun des quatre plannings PDF
(public du site : personnels administratifs). Il reçoit le public « Personnels », avec
sa bulle, qui n'apparaît que si une séance au moins le porte : sans cette valeur dans
la colonne Cibles, la rangée garde ses quatre bulles et le rendu est inchangé.

- widget.js : public « Personnels » (dernier de la rangée), lu avec ou sans accent.
- data/build_xlsx.py : « Personnels » sur cette seule séance ; « tous » reste les quatre plannings.
- Tests : option ?sans-personnels du faux Grist, filtre Personnels (faux et vrai Grist,
  valeur hors liste de choix comprise), lecture des valeurs.
- README et numéro de version à jour.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FPLB4wrip8pBNBGYDq5d2D
</commit_message>
<xml_diff>
--- a/data/Evenements_Semaine_Innovation_2026.xlsx
+++ b/data/Evenements_Semaine_Innovation_2026.xlsx
@@ -2338,7 +2338,11 @@
           <t>Personnels administratifs</t>
         </is>
       </c>
-      <c r="L30" s="5" t="n"/>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>Personnels</t>
+        </is>
+      </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
           <t>Jeu en équipes de 4 à 5 personnes pour tester sa connaissance de l’écosystème d’innovation bordelais et savoir orienter les porteurs de projets.</t>

</xml_diff>